<commit_message>
RF-26 panel actualizacion masiva: limite/offset/depto + polling 1s + ultima actualizacion + fix sin fecha
</commit_message>
<xml_diff>
--- a/SECOP_Backlog_Producto.xlsx
+++ b/SECOP_Backlog_Producto.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2714,6 +2714,370 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>RF-29</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero entrar por la pagina /login con correo y contrasena para usar el dashboard sin pegar tokens a mano.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>RF-04</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>3 horas</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Formulario React en /login -&gt; POST /api/auth/login/ guarda access+refresh en localStorage y va a /; sin token / redirige a /login; boton Salir invalida refresh (best-effort) + limpia local. Routing por pathname sin React Router.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>RF-30</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero recuperar mi clave desde /recuperar y /restablecer para volver a entrar sin ayuda del administrador.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>RF-22</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2 horas</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>/recuperar pide correo -&gt; POST /api/auth/recuperar/ siempre 200 sin revelar; /restablecer?token= pide nueva con politica 8+ may/min/num -&gt; POST /api/auth/restablecer/; enlace 30min 1 solo uso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>RF-31</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero ver el dashboard con KPIs y filtros combinables para entender el gasto sin recargar la pagina.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>RF-12</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>4 horas</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Dashboard.jsx con TanStack Query queryKey [resumen,depto] enabled !!token cache 5min, placeholderData keepPreviousData para no desmontar Leaflet, skeleton solo si cargando y sin datos, header role banner main#contenido skip-link aria-live polite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>RF-32</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero una tabla rapida con boton CSV para revisar miles de contratos sin que se congele y descargar lo filtrado.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>RF-11</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2 horas</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>useVirtualizer estimateSize 44 overscan 8 sobre filas paginadas (~16 en DOM), paginacion 20/page, boton CSV descarga filtro actual con BOM UTF-8, vacio solo cabecera, error 503 muestra detalle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>RF-33</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero un mapa clicable y un buscador tipo Google para filtrar por territorio o texto sin perder mis filtros.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>RF-15</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>4 horas</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>MapaDirecta.jsx Leaflet POR_ID 33 colorFor papel-&gt;rojo tooltip monto/% fitBounds clic filtra y VER TODO limpia; Buscador debounce 300ms abort icontains agrupado 10/grupo con highlight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>RF-34</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero ver alertas y lista de entidades con umbrales editables para ajustar la deteccion sin reiniciar.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>RF-19</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>3 horas</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Banderas concentracion X=30% tabla roja, Predominio directa X=80% tabla amarilla, Umbrales panel Guarda y recalcula sin reinicio persiste en umbral_alerta, Entidades buscador nombre/NIT paginado clic muestra totales/modalidad/top, sin contratos dice 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>RF-35</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero una red entidad-&gt;contratista navegable con teclado para detectar concentracion visualmente.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>RF-17</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>3 horas</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Grafo.jsx react-force-graph nodo verde entidad azul contratista arista grosor por monto color por modalidad (roja directa verde licitacion) zoom/drag, contraste 7:1 focus 2px #059669 skip-link, browserslist last 2, dist minificado.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2726,7 +3090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4152,6 +4516,242 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>RF-29</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero entrar por la pagina /login con correo y contrasena para usar el dashboard sin pegar tokens a mano.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>1. DADO que no hay token CUANDO abre / ENTONCES redirige a /login
+2. DADO credenciales validas CUANDO envia ENTONCES guarda tokens y va a /
+3. DADO clic en Salir CUANDO sale ENTONCES limpia local y refresh queda invalidado
+4. DADO token vencido CUANDO consulta ENTONCES responde 401 y vuelve a /login</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1. Permite entrar a / sin token
+2. Guarda la contrasena en localStorage
+3. No limpia tokens al salir
+4. No muestra error con credenciales invalidas</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>RF-30</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero recuperar mi clave desde /recuperar y /restablecer para volver a entrar sin ayuda del administrador.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1. Solicitar con correo existente devuelve 200 y crea token 32 hex
+2. Restablecer con token valido devuelve 200 y login con nueva da 200
+3. Reuso del mismo enlace devuelve 400 ya utilizado
+4. Enlace expirado 30min devuelve 400 expirado
+5. Correo inexistente devuelve 200 sin crear enlace</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1. Revela si el correo existe
+2. Permite reusar el enlace mas de una vez
+3. Acepta clave debil sin may/min/num
+4. No lee el parametro ?token= de la URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>RF-31</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero ver el dashboard con KPIs y filtros combinables para entender el gasto sin recargar la pagina.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1. KPIs total dinero/total/promedio se recalculan al cambiar filtro
+2. Filtros depto/modalidad/fechas son combinables y persisten
+3. Clic en mapa no destruye la pagina (keepPreviousData)
+4. Muestra skeleton solo en primera carga, no en cada filtro
+5. Tab recorre select-&gt;boton-&gt;tabla-&gt;mapa sin raton</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1. Early return if(cargando) desmonta el mapa y pierde zoom
+2. Filtros se pierden al navegar entre vistas
+3. KPIs muestran valores viejos del filtro anterior
+4. Sin skeleton ni aria-live en carga</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>RF-32</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero una tabla rapida con boton CSV para revisar miles de contratos sin que se congele y descargar lo filtrado.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>1. Scroll mantiene 60FPS con max 50 nodos en DOM
+2. Paginacion 20/page con next/previous/count
+3. Exportar abre en Excel con tildes y punto decimal
+4. Filtro vacio exporta solo cabecera sin error</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1. Renderiza todas las filas al DOM y se congela
+2. Exporta datos globales ignorando el filtro
+3. CSV sin BOM muestra caracteres raros
+4. Export vacio devuelve error en vez de cabecera</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>RF-33</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero un mapa clicable y un buscador tipo Google para filtrar por territorio o texto sin perder mis filtros.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>1. Mapa pinta escala continua y tooltip con monto+%
+2. Clic en territorio refiltra KPIs sin borrar otros filtros
+3. Buscador no dispara por tecla sin debounce 300ms
+4. Cancela peticiones viejas y agrupa 10/grupo
+5. Busqueda sin coincidencias devuelve vacio sin error</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1. Mapa beige vacio sin colores
+2. Clic recarga la pagina o borra filtros
+3. Dispara peticion por cada tecla sin debounce
+4. Respuesta vieja sobrescribe a la nueva (race condition)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>RF-34</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero ver alertas y lista de entidades con umbrales editables para ajustar la deteccion sin reiniciar.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>1. Umbrales listan valores actuales y validan rango 400 si invalido
+2. Cambio de umbral recalcula sin reinicio
+3. Entidades buscan por nombre/NIT y paginan
+4. Clic en entidad muestra totales y top contratistas
+5. Entidad sin contratos devuelve 0 sin error</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1. Umbral fijo no configurable
+2. Cambio exige reinicio manual
+3. Entidades sin paginacion traen todo de una vez
+4. Entidad sin contratos devuelve error</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>RF-35</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero una red entidad-&gt;contratista navegable con teclado para detectar concentracion visualmente.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1. Grafo permite zoom/drag y destaca NIT sobre umbral
+2. Arista grosor por monto y color por modalidad
+3. Tab recorre toda la interfaz sin raton con foco visible
+4. Funciona en Chrome/Firefox/Edge/Safari sin errores consola
+5. Build minificado OK</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>1. Grafo estatico sin zoom ni drag
+2. Todas las aristas igual grosor y color
+3. Sin foco visible al navegar con teclado
+4. Solo funciona en un navegador</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(auditoria): informe 2026-09-18 + migracion 0010 + Radares SaaS + DashboardModern OLED + backlog 56 historias
</commit_message>
<xml_diff>
--- a/SECOP_Backlog_Producto.xlsx
+++ b/SECOP_Backlog_Producto.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +34,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +58,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00EAF1F8"/>
         <bgColor rgb="00EAF1F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A3C5E"/>
+        <bgColor rgb="001A3C5E"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -97,6 +109,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -463,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -479,52 +494,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Requisito</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Historia de Usuario</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Dependencia</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Prioridad</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Estimación</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Encargado</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Tiempo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Regla de negocio</t>
         </is>
@@ -583,52 +598,52 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>RF-25</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero crear un modelo separado de Entidad con sus propios atributos para analizar la contratación a nivel de la entidad de forma más rigurosa.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>5 horas</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>El modelo Entidad debe ser una tabla independiente con atributos como nombre_entidad, nit_entidad, departamento, ciudad y sector. El modelo Contrato debe relacionarse a Entidad mediante una clave foránea. Su creación ocurre en el mismo sprint que el modelo Contrato, ya que la relación se define desde el diseño de esquema.</t>
         </is>
@@ -687,52 +702,52 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero registrarme en la plataforma con correo y contraseña para crear una cuenta de acceso al sistema.</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Ninguna</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>5 horas</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>El correo debe ser único y válido en formato estándar. La contraseña debe cumplir mínimo 8 caracteres con al menos una mayúscula, una minúscula y un número, y debe almacenarse con algoritmo PBKDF2. El endpoint de registro debe responder HTTP 201 y validar los datos con serializers.</t>
         </is>
@@ -791,52 +806,52 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero cerrar sesión para invalidar mi token de acceso y proteger mi cuenta.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>2.5 horas</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>El endpoint de logout debe revocar la sesión actual. El token de acceso debe invalidarse antes de su expiración natural. Tras el logout, cualquier petición protegida con ese token debe responder HTTP 401.</t>
         </is>
@@ -895,52 +910,52 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>RNF-02</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo disponer de las variables de configuración separadas del código para funcionar en distintos entornos sin exponer secretos.</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Toda configuración sensible (token de acceso a datos, credenciales de base de datos, clave JWT) debe leerse de variables de entorno. Debe entregarse un archivo .env.example con claves vacías; el .env nunca debe versionarse. Los entornos de desarrollo y producción deben usar valores independientes.</t>
         </is>
@@ -999,52 +1014,52 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero monitorear el progreso de una ingesta en curso para saber cuándo termina y detectar errores.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>4 horas</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>El endpoint GET /api/jobs/{id}/ debe devolver JSON con id, estado, progress y mensaje de error. La ingesta debe ejecutarse en un hilo en segundo plano para no bloquear la petición. El endpoint de inicio POST /api/sincronizar/ debe responder HTTP 202 Accepted de inmediato.</t>
         </is>
@@ -1103,52 +1118,52 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>RF-09</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero consultar el top de contratistas por monto contratado para identificar los mayores receptores de contratación en un territorio.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>4 horas</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>El endpoint GET /api/top-contratistas debe agrupar por contratista_nit con GROUP BY, ordenado descendente por SUM(valor_contrato), limitando a 10 resultados. Debe devolver contratista_nit, contratista_nombre y total_contratado.</t>
         </is>
@@ -1207,52 +1222,52 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>RF-11</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero consultar la lista de contratos paginada para navegar por los registros sin cargar todos a la vez.</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>4 horas</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>El endpoint GET /api/contratos?page=N debe devolver un máximo de 50 registros por página con metadatos next, previous, count y total_pages. Si page está fuera de rango debe responder HTTP 400. Los registros deben devolverse agregados, nunca el dataset completo.</t>
         </is>
@@ -1311,52 +1326,52 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>RNF-04</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo validar la calidad de los datos durante la ingesta para evitar registros corruptos en la base de datos.</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Durante la transformación, valor_contrato debe convertirse de texto a Decimal descartando los que no sean numéricos. Las filas inválidas deben registrarse en un log sin abortar toda la ingesta. Los registros con duplicados por id_contrato deben omitirse sin duplicar la carga.</t>
         </is>
@@ -1415,52 +1430,52 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>RNF-06</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo limitar la cantidad de peticiones al API para proteger el servicio de abusos y sobrecarga.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>1.5 horas</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Se debe implementar límite de peticiones usando Django Rest Framework throttling. El límite debe ser de 60 peticiones por minuto por usuario para endpoints de consulta. Al superar el límite debe responder HTTP 429 con el tiempo de espera en segundos.</t>
         </is>
@@ -1519,52 +1534,52 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver un dashboard con indicadores clave del gasto público para tener una visión general de la contratación.</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>RF-08</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>6.5 horas</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>El dashboard debe mostrar KPIs de total de dinero, total de contratos y valor promedio, más una tabla virtualizada de contratos que renderice solo las filas visibles usando virtualización de react. El estado del dashboard debe sincronizarse con la caché de datos del cliente.</t>
         </is>
@@ -1623,52 +1638,52 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>RF-14</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver la serie mensual de contratación para observar la tendencia del gasto a lo largo del tiempo.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>3 horas</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>El endpoint GET /api/serie-mensual debe agrupar por periodo mensual con DATE_TRUNC y devolver suma de valor_contrato y conteo de contratos ordenados cronológicamente. Debe renderizarse en un gráfico de línea.</t>
         </is>
@@ -1727,52 +1742,52 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>RF-16</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero seleccionar un territorio del mapa para actualizar todos los indicadores del dashboard a ese territorio y profundizar su análisis.</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>RF-15</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>3.5 horas</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Al seleccionar un territorio, el filtro global debe actualizarse y re-consultar los KPIs, gráficos y tabla. El territorio seleccionado debe resaltarse visualmente en el mapa y el filtro debe combinarse con los demás filtros activos.</t>
         </is>
@@ -1831,52 +1846,52 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>RNF-07</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo mantener una interfaz fluida a 60 cuadros por segundo para no degradar la experiencia con grandes volúmenes de datos.</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Las tablas con grandes volúmenes deben usar virtualización para renderizar solo las filas visibles (máximo 50 nodos en el DOM). Las consultas deben cachearse en el cliente para evitar repeticiones. La renderización de la interfaz no debe bajar de 60 cuadros por segundo.</t>
         </is>
@@ -1935,52 +1950,52 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>RNF-14</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo ser mantenible mediante patrones de diseño y desacoplamiento para facilitar los cambios futuros.</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>RF-01</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>El backend debe estructurarse en módulos con responsabilidades separadas: modelos, serializadores, vistas y lógica de ingesta. El acceso a datos debe centralizarse para que un cambio de fuente o de motor de base de datos no implique reescribir las vistas. El código debe seguir un estándar de estilo definido y verificable.</t>
         </is>
@@ -2039,52 +2054,52 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>RF-19</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver alertas de banderas rojas de concentración de contratación para detectar posibles irregularidades en el gasto público.</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>RF-13</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Se debe marcar con bandera roja un contratista que concentre más de un porcentaje configurable del presupuesto de una entidad en un periodo configurable. Debe mostrar el contratista, la entidad, el porcentaje de concentración y el monto. El umbral debe ser configurable por el administrador.</t>
         </is>
@@ -2143,52 +2158,52 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>RF-21</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero exportar los resultados de un análisis a un archivo para compartir la información con otros interesados.</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>RF-13</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>El endpoint de exportación debe generar un archivo CSV con codificación UTF-8 con BOM que abra correctamente en Excel. La exportación debe respetar el conjunto de datos filtrado actualmente. Los valores numéricos deben expresarse con separador decimal de punto.</t>
         </is>
@@ -2247,52 +2262,52 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>RF-23</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero gestionar el catálogo de datos y monitorear los procesos mediante un panel de administración para mantener la plataforma sin escribir SQL.</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>3 horas</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>El panel de administración debe permitir gestionar los modelos de contrato y de proceso de ingesta, mostrar el estado y progreso de cada ingesta y auditar los registros cargados. No es el producto principal sino una herramienta de soporte, por lo que se ubica en el sprint final.</t>
         </is>
@@ -2351,52 +2366,52 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>RF-26</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero programar la actualización periódica de los datos de contratación para mantener la información al día sin intervención manual.</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>RF-06</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>5 horas</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J37" s="3" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>La actualización debe permitir ejecutarse de forma periódica reutilizando la lógica de ingesta paginada, sin duplicar registros ya existentes mediante la detección por id_contrato. Debe existir un mecanismo para registrar la fecha y hora de la última actualización y el estado de la misma.</t>
         </is>
@@ -2455,52 +2470,52 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>RF-28</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver una lista de todas las entidades con su información para explorar el catálogo de entidades de contratación.</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>RF-25</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="H39" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>El endpoint GET /api/entidades debe devolver el listado paginado de entidades con nombre, NIT, departamento, ciudad y sector. Debe ordenarse por nombre y permitir búsqueda por nombre o NIT. Debe requerir paginación con un máximo de 100 registros por página.</t>
         </is>
@@ -2559,52 +2574,52 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>RNF-10</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo desplegarse de forma reproducible y documentada para reducir errores de configuración en producción.</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>RF-02</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="H41" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I41" s="3" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J41" s="3" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>El despliegue debe realizarse en proveedores de nube para la base de datos, el backend y el frontend, todos usando HTTPS. Debe existir documentación de despliegue con pasos reproducibles. Las migraciones deben aplicarse antes de publicar el código, y el proceso debe ser el descrito por las variables de entorno.</t>
         </is>
@@ -2663,418 +2678,782 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>RNF-12</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo ser compatible con los navegadores modernos principales para permitir el acceso de la mayoría de usuarios.</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Por asignar</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr">
+      <c r="H43" s="4" t="inlineStr">
         <is>
           <t>1 hora</t>
         </is>
       </c>
-      <c r="I43" s="3" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
         <is>
           <t>El frontend debe funcionar correctamente en las últimas versiones de los navegadores principales. Debe emplearse JavaScript moderno compatible y el código de producción debe estar optimizado y minificado para reducir tiempo de carga.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>RF-29</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero entrar por la pagina /login con correo y contrasena para usar el dashboard sin pegar tokens a mano.</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>RF-04</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Steven Araque</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>3 horas</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>Formulario React en /login -&gt; POST /api/auth/login/ guarda access+refresh en localStorage y va a /; sin token / redirige a /login; boton Salir invalida refresh (best-effort) + limpia local. Routing por pathname sin React Router.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>RF-30</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero recuperar mi clave desde /recuperar y /restablecer para volver a entrar sin ayuda del administrador.</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>RF-22</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>Steven Araque</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>2 horas</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>/recuperar pide correo -&gt; POST /api/auth/recuperar/ siempre 200 sin revelar; /restablecer?token= pide nueva con politica 8+ may/min/num -&gt; POST /api/auth/restablecer/; enlace 30min 1 solo uso.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>RF-31</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver el dashboard con KPIs y filtros combinables para entender el gasto sin recargar la pagina.</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Steven Araque</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" s="4" t="inlineStr">
         <is>
           <t>4 horas</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>Dashboard.jsx con TanStack Query queryKey [resumen,depto] enabled !!token cache 5min, placeholderData keepPreviousData para no desmontar Leaflet, skeleton solo si cargando y sin datos, header role banner main#contenido skip-link aria-live polite.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>RF-32</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero una tabla rapida con boton CSV para revisar miles de contratos sin que se congele y descargar lo filtrado.</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>RF-11</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Steven Araque</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>2 horas</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>useVirtualizer estimateSize 44 overscan 8 sobre filas paginadas (~16 en DOM), paginacion 20/page, boton CSV descarga filtro actual con BOM UTF-8, vacio solo cabecera, error 503 muestra detalle.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>RF-33</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero un mapa clicable y un buscador tipo Google para filtrar por territorio o texto sin perder mis filtros.</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>RF-15</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Steven Araque</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>4 horas</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
         <is>
           <t>MapaDirecta.jsx Leaflet POR_ID 33 colorFor papel-&gt;rojo tooltip monto/% fitBounds clic filtra y VER TODO limpia; Buscador debounce 300ms abort icontains agrupado 10/grupo con highlight.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>RF-34</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver alertas y lista de entidades con umbrales editables para ajustar la deteccion sin reiniciar.</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>RF-19</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>Steven Araque</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H49" s="4" t="inlineStr">
         <is>
           <t>3 horas</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>Banderas concentracion X=30% tabla roja, Predominio directa X=80% tabla amarilla, Umbrales panel Guarda y recalcula sin reinicio persiste en umbral_alerta, Entidades buscador nombre/NIT paginado clic muestra totales/modalidad/top, sin contratos dice 0.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>RF-35</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero una red entidad-&gt;contratista navegable con teclado para detectar concentracion visualmente.</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>RF-17</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Steven Araque</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>3 horas</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
         <is>
           <t>Grafo.jsx react-force-graph nodo verde entidad azul contratista arista grosor por monto color por modalidad (roja directa verde licitacion) zoom/drag, contraste 7:1 focus 2px #059669 skip-link, browserslist last 2, dist minificado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>RF-36</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero crear un Radar con departamento objetivo, palabras clave y rango de cuantia para guardar mi preferencia de busqueda y recibir oportunidades automaticas.</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>RF-04</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>4 horas</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>El Radar debe persistirse con usuario FK, departamento_objetivo, palabras_clave, rango_cuantia_min/max Decimal(18,2), activo bool. Debe validarse palabras_clave no vacias y rango_min &lt;= rango_max. Endpoint POST /api/radares/ con IsAuthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>RF-37</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero listar mis Radares para ver y gestionar mis preferencias guardadas.</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>RF-36</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>2 horas</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/radares/ debe devolver solo radares del usuario autenticado, paginados, ordenados por creado_en desc. Debe requerir JWT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>RF-38</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero actualizar o eliminar un Radar para ajustar mis intereses sin crear uno nuevo.</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>RF-37</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>2 horas</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>PUT/PATCH /api/radares/{id}/ y DELETE deben validar pertenencia al usuario (404 si no es suyo). Validar mismo que en creacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>RF-39</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero consultar mi bandeja privada de Oportunidades (mis matches) para ver contratos que coinciden con mis Radares sin buscar manualmente.</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>RF-36</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Yesid Amaya</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>5 horas</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>GET /api/mis-oportunidades/ debe devolver Oportunidades del usuario via sus Radares, con contrato embebido, estado Nueva/Guardada/Postulado, paginada. Solo IsAuthenticated. Generadas por matchmaking post-ETL via ILIKE + rango + depto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>RF-40</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero marcar una Oportunidad como Guardada o Postulada para organizar mi flujo de trabajo.</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>RF-39</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Yesid Amaya</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>2 horas</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/mis-oportunidades/{id}/ con estado Guardada/Postulado debe validar pertenencia via radar.usuario. Estados validos solo esos tres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>RF-41</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero recibir un email cuando se cree una nueva Oportunidad que coincide con mi Radar para no revisar la bandeja a diario.</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>RF-39</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Yesid Amaya</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>3 horas</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Tras bulk_create Oportunidad, el sistema debe enviar email via send_mail a usuario.email con asunto y link a /app. En dev console backend, en prod SMTP via .env. No debe bloquear ETL si falla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>RF-42</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero poder filtrar y crear Radares usando cualquiera de las 85 columnas del dataset (filtros elegibles) para precisar mi busqueda mas alla de depto y palabras clave.</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>RF-36</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Steven Araque</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>4 horas</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Radar debe permitir filtros elegibles sobre cualquier de las 85 columnas (departamento, modalidad, estado, ciudad, sector, etc.). Validacion: campo debe existir en modelo Contrato y valor debe ser del tipo correcto. Endpoint debe construir Q objects dinamicos.</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3101,27 +3480,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Requisito</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Historia de Usuario</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Criterios de Aceptación</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Criterios de Rechazo</t>
         </is>
@@ -3162,22 +3541,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>RF-25</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero crear un modelo separado de Entidad con sus propios atributos para analizar la contratación a nivel de la entidad de forma más rigurosa.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe crear el modelo Entidad como tabla independiente con atributos nombre_entidad, nit_entidad, departamento, ciudad y sector
 2. El sistema debe relacionar el modelo Contrato a Entidad mediante una clave foránea
@@ -3185,7 +3564,7 @@
 4. DADO que un contrato se asocia a una entidad, CUANDO se consulta, ENTONCES el análisis puede agrupar por esta entidad</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>1. El modelo Entidad no existe como tabla propia y queda como campo de texto dentro de Contrato
 2. La relación entre Contrato y Entidad no se define mediante clave foránea
@@ -3228,22 +3607,22 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>RF-03</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero registrarme en la plataforma con correo y contraseña para crear una cuenta de acceso al sistema.</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>1. DADO que el usuario ingresa un correo nuevo y una contraseña que cumple la política, CUANDO envía el formulario de registro, ENTONCES el sistema responde HTTP 201 y crea la cuenta
 2. DADO que el usuario ingresa un correo ya registrado, CUANDO envía el formulario, ENTONCES el sistema responde HTTP 400 indicando que el correo ya existe
@@ -3252,7 +3631,7 @@
 5. DADO que el usuario ingresa el campo de correo con formato inválido (sin @ o sin dominio), CUANDO envía el formulario, ENTONCES el sistema responde HTTP 400</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>1. El sistema responde 201 pero almacena la contraseña en texto plano o con hash débil distinto a PBKDF2
 2. El sistema responde 201 con un correo duplicado, permitiendo dos cuentas con el mismo correo
@@ -3295,22 +3674,22 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>RF-05</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero cerrar sesión para invalidar mi token de acceso y proteger mi cuenta.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>1. DADO que el usuario está autenticado, CUANDO solicita cerrar sesión, ENTONCES el sistema responde HTTP 200 y el token de acceso queda invalidado
 2. DADO que el usuario cierra sesión, CUANDO intenta acceder a un endpoint protegido con el token revocado, ENTONCES el sistema responde HTTP 401
@@ -3318,7 +3697,7 @@
 4. DADO que el usuario cierra sesión con un token de refresco asociado, CUANDO se cierra la sesión, ENTONCES el token de refresco también se revoca y no puede usarse para obtener un nuevo access token</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>1. El sistema responde 200 pero el token sigue siendo válido después del cierre de sesión
 2. El sistema permite al usuario reutilizar el token revocado para acceder a datos protegidos
@@ -3360,22 +3739,22 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>RNF-02</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo disponer de las variables de configuración separadas del código para funcionar en distintos entornos sin exponer secretos.</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe leer toda la configuración sensible (token de acceso a datos, credenciales de base de datos, clave JWT) de variables de entorno, nunca de código
 2. El sistema debe incluir un archivo .env.example con las claves de configuración vacías y documentadas
@@ -3383,7 +3762,7 @@
 4. El sistema debe permitir configurar valores independientes para los entornos de desarrollo y producción</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>1. El archivo .env se versiona y queda expuesto con credenciales reales en el repositorio
 2. Una credencial sensible (como la clave JWT) está hardcodeada en el código fuente
@@ -3427,22 +3806,22 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>RF-07</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero monitorear el progreso de una ingesta en curso para saber cuándo termina y detectar errores.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>1. DADO que hay una ingesta en curso, CUANDO el usuario consulta el estado del job, ENTONCES el sistema devuelve el estado, el progreso numérico y el mensaje de error en JSON
 2. DADO que el usuario inicia una ingesta, CUANDO envía la petición, ENTONCES el sistema responde HTTP 202 Accepted de inmediato sin bloquear
@@ -3450,7 +3829,7 @@
 4. DADO que el job termina, CUANDO se consulta, ENTONCES devuelve el estado completed y el progreso 100</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>1. El sistema bloquea la petición de inicio hasta que termina toda la ingesta
 2. El estado del job se queda en running aunque el proceso terminó o falló
@@ -3494,22 +3873,22 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>RF-09</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero consultar el top de contratistas por monto contratado para identificar los mayores receptores de contratación en un territorio.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>1. DADO que el usuario consulta el top de contratistas, CUANDO se ejecuta la consulta, ENTONCES el sistema devuelve los 10 contratistas con mayor monto contratado agrupados por contratista_nit
 2. El sistema debe agrupar por contratista_nit con GROUP BY y ordenar descendente por la suma del monto contratado
@@ -3518,7 +3897,7 @@
 5. DADO que el usuario filtra por departamento, CUANDO consulta el top, ENTONCES el ranking se calcula dentro de ese territorio</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1. El sistema devuelve más de 10 contratistas en el top sin aplicar el límite
 2. El ranking no está ordenado por monto contratado, mostrando los contratistas en orden arbitrario
@@ -3561,22 +3940,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>RF-11</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero consultar la lista de contratos paginada para navegar por los registros sin cargar todos a la vez.</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>1. DADO que el usuario solicita la lista de contratos con un número de página, CUANDO ejecuta la consulta, ENTONCES el sistema devuelve máximo 50 registros más los metadatos next, previous, count y total_pages
 2. DADO que el usuario solicita una página fuera de rango, CUANDO ejecuta la consulta, ENTONCES el sistema responde HTTP 400
@@ -3584,7 +3963,7 @@
 4. DADO que la lista está vacía para los filtros aplicados, CUANDO se consulta, ENTONCES el sistema devuelve count=0 y lista vacía sin error</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>1. El sistema devuelve todos los registros de una vez ignorando la paginación
 2. El metadato total_pages es incorrecto respecto al total de registros
@@ -3627,22 +4006,22 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>RNF-04</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo validar la calidad de los datos durante la ingesta para evitar registros corruptos en la base de datos.</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>1. Durante la transformación de ingesta, el sistema debe convertir valor_contrato de texto a valor numérico descartando los registros que no sean numéricos
 2. El sistema debe registrar las filas inválidas en un log sin abortar toda la ingesta por errores parciales
@@ -3650,7 +4029,7 @@
 4. DADO que una fila tiene un campo faltante requerido, CUANDO se procesa, ENTONCES la fila se registra como inválida y el proceso continúa</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>1. El sistema aborta toda la ingesta ante el primer registro inválido
 2. Un registro con valor_contrato no numérico se inserta en la base de datos sin corrección
@@ -3692,29 +4071,29 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>RNF-06</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo limitar la cantidad de peticiones al API para proteger el servicio de abusos y sobrecarga.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe limitar la cantidad de peticiones de los endpoints de consulta usando un mecanismo de throttling del framework
 2. DADO que un usuario excede el límite de 60 peticiones por minuto, CUANDO continúa consultando, ENTONCES el sistema responde HTTP 429 con el tiempo de espera en segundos
 3. DADO que el usuario está dentro del límite, CUANDO consulta, ENTONCES el sistema responde normalmente sin error de límite</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>1. El sistema permite más de 60 peticiones por minuto sin bloquear al usuario
 2. El sistema responde error de límite (429) sin indicar el tiempo de espera restante
@@ -3756,22 +4135,22 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>RF-12</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver un dashboard con indicadores clave del gasto público para tener una visión general de la contratación.</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe mostrar en el dashboard los indicadores clave: total de dinero, total de contratos y valor promedio
 2. El sistema debe renderizar una tabla virtualizada que solo muestre las filas visibles en pantalla y mantenga la fluidez
@@ -3779,7 +4158,7 @@
 4. El sistema debe sincronizar el estado del dashboard con la caché de datos del cliente para evitar consultas duplicadas</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>1. Los KPIs muestran valores desactualizados respecto a los datos aplicando los filtros actuales
 2. La tabla carga todas las filas al DOM y el dashboard se vuelve lento o no responde a 60 cuadros
@@ -3822,22 +4201,22 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>RF-14</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver la serie mensual de contratación para observar la tendencia del gasto a lo largo del tiempo.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe devolver la suma de valor_contrato y el conteo de contratos agrupados por periodo mensual, ordenados cronológicamente
 2. DADO que existen contratos en varios meses consecutivos, CUANDO se consulta la serie, ENTONCES se devuelven todos los periodos con sus valores
@@ -3845,7 +4224,7 @@
 4. El sistema debe renderizar la serie en un gráfico de línea para visualizar la tendencia</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>1. La serie devuelve meses fuera de orden cronológico
 2. Los valores mensuales no coinciden con la sumatoria de los contratos de ese mes
@@ -3888,22 +4267,22 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>RF-16</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero seleccionar un territorio del mapa para actualizar todos los indicadores del dashboard a ese territorio y profundizar su análisis.</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>1. DADO que el usuario hace clic en un territorio del mapa, CUANDO lo selecciona, ENTONCES el filtro global se actualiza a ese territorio
 2. DADO que se selecciona un territorio, CUANDO se actualizan los indicadores, ENTONCES los KPIs, gráficos y tabla se recomputan con ese territorio
@@ -3911,7 +4290,7 @@
 4. DADO que hay otros filtros activos, CUANDO se selecciona un territorio, ENTONCES el filtro se combina con los demás sin sustituirlos</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>1. Al hacer clic en un territorio el mapa cambia de color pero los datos del dashboard no se actualizan
 2. El territorio seleccionado no se resalta, no se distingue del resto
@@ -3955,29 +4334,29 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>RNF-07</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo mantener una interfaz fluida a 60 cuadros por segundo para no degradar la experiencia con grandes volúmenes de datos.</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe renderizar las tablas con grandes volúmenes usando virtualización, mostrando máximo 50 filas en el DOM
 2. El sistema debe cachear las consultas en el cliente mediante la gestión de estado del frontend para evitar repeticiones
 3. DADO que se interactúa con la tabla o los gráficos sobre un conjunto de al menos 50000 registros, CUANDO se desplaza o actualiza la vista, ENTONCES el tiempo entre fotogramas no supera 16.67 milisegundos (equivalente a 60 cuadros por segundo), medido con la herramienta de análisis de rendimiento del navegador durante una interacción sostenida de 30 segundos</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>1. La tabla renderiza todas las filas al DOM superando los 50 nodos visibles
 2. Las interacciones del dashboard caen por debajo de 60 cuadros por segundo con datos grandes
@@ -4020,22 +4399,22 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>RNF-14</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo ser mantenible mediante patrones de diseño y desacoplamiento para facilitar los cambios futuros.</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>1. El backend debe estructurarse en módulos con responsabilidades separadas: modelos, serializadores, vistas y lógica de ingesta
 2. El acceso a datos debe centralizarse para que un cambio de fuente o de motor de base de datos no implique reescribir las vistas
@@ -4043,7 +4422,7 @@
 4. DADO que se requiere un cambio en la fuente de datos, CUANDO se modifica, ENTONCES solo se afecta el módulo correspondiente sin tocar las vistas</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>1. La lógica de ingesta, vista y serialización está mezclada en un solo archivo sin separación
 2. Un cambio de fuente de datos obliga a reescribir las vistas del API
@@ -4086,22 +4465,22 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>RF-19</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver alertas de banderas rojas de concentración de contratación para detectar posibles irregularidades en el gasto público.</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe marcar con bandera roja un contratista que concentre más de un porcentaje configurable del presupuesto de una entidad en un periodo configurable
 2. El sistema debe mostrar la alerta con el contratista, la entidad, el porcentaje de concentración y el monto involucrado
@@ -4110,7 +4489,7 @@
 5. DADO que el umbral se modifica, CUANDO se vuelven a evaluar los datos, ENTONCES las banderas rojas se recalculan según el nuevo umbral</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>1. El sistema marca banderas rojas con un umbral fijo que no puede configurarse
 2. La alerta no muestra el porcentaje de concentración ni el monto
@@ -4153,22 +4532,22 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>RF-21</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero exportar los resultados de un análisis a un archivo para compartir la información con otros interesados.</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe generar un archivo CSV que respete el conjunto de datos filtrado actualmente
 2. El archivo CSV debe usar codificación UTF-8 con BOM para que los caracteres especiales se abran correctamente en Excel
@@ -4176,7 +4555,7 @@
 4. DADO que no hay datos que coincidan con los filtros, CUANDO se exporta, ENTONCES el sistema genera el archivo con solo la cabecera sin error</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>1. El CSV se abre en Excel mostrando caracteres extraños por falta de BOM
 2. El archivo exporta datos globales en lugar del resultado filtrado actual
@@ -4220,22 +4599,22 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>RF-23</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero gestionar el catálogo de datos y monitorear los procesos mediante un panel de administración para mantener la plataforma sin escribir SQL.</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe permitir administrar los modelos de contrato y de proceso de ingesta mediante el panel de administración sin escribir SQL
 2. El panel de administración debe mostrar el estado y el progreso de cada ingesta
@@ -4243,7 +4622,7 @@
 4. El panel es una herramienta de soporte accesible únicamente por el administrador autenticado</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>1. El panel de administración no muestra el estado ni el progreso de las ingestas
 2. Usuarios sin permisos de administrador pueden acceder al panel
@@ -4286,22 +4665,22 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>RF-26</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Como administrador del sistema, quiero programar la actualización periódica de los datos de contratación para mantener la información al día sin intervención manual.</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe permitir ejecutar la actualización de datos de forma periódica reutilizando la lógica de ingesta paginada
 2. El sistema debe evitar duplicar registros existentes durante la actualización detectando los ya cargados por id_contrato
@@ -4309,7 +4688,7 @@
 4. DADO que una actualización está en curso, CUANDO se evalúa, ENTONCES el estado se registra coherentemente y no se mezcla con datos de otra actualización</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>1. Una actualización periódica duplica los registros ya existentes
 2. El sistema no reutiliza la lógica de ingesta y reimplementa la carga por separado
@@ -4352,22 +4731,22 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>RF-28</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver una lista de todas las entidades con su información para explorar el catálogo de entidades de contratación.</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe devolver el listado paginado de entidades con nombre, NIT, departamento, ciudad y sector
 2. El sistema debe ordenar el listado por nombre de entidad
@@ -4376,7 +4755,7 @@
 5. DADO que se solicita una página fuera de rango, CUANDO se consulta, ENTONCES el sistema responde HTTP 400</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>1. El listado de entidades no está paginado y devuelve todas de una vez
 2. El sistema no permite buscar por nombre o NIT de la entidad
@@ -4418,22 +4797,22 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>RNF-10</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo desplegarse de forma reproducible y documentada para reducir errores de configuración en producción.</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe desplegarse en proveedores de nube para la base de datos, el backend y el frontend, todos usando HTTPS
 2. El sistema debe contar con documentación de despliegue con pasos reproducibles
@@ -4441,7 +4820,7 @@
 4. Los valores de configuración por entorno deben provenir de variables de entorno separadas por entorno</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>1. El despliegue se realiza sin HTTPS en alguno de los componentes
 2. Las migraciones se aplican después de publicar el código, rompiendo el esquema en producción
@@ -4484,22 +4863,22 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>RNF-12</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>NF</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Como sistema, debo ser compatible con los navegadores modernos principales para permitir el acceso de la mayoría de usuarios.</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>1. El sistema debe funcionar correctamente en las últimas versiones de los principales navegadores (Chrome, Firefox, Edge, Safari)
 2. El sistema debe emplear JavaScript moderno compatible con los navegadores soportados
@@ -4507,7 +4886,7 @@
 4. DADO que el usuario abre la interfaz en uno de los navegadores soportados, CUANDO la usa, ENTONCES todas las funciones principales operan sin errores de consola</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>1. La interfaz no funciona en alguno de los navegadores principales soportados
 2. El bundle de producción no está minificado, aumentando el tiempo de carga
@@ -4517,22 +4896,22 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>RF-29</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero entrar por la pagina /login con correo y contrasena para usar el dashboard sin pegar tokens a mano.</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>1. DADO que no hay token CUANDO abre / ENTONCES redirige a /login
 2. DADO credenciales validas CUANDO envia ENTONCES guarda tokens y va a /
@@ -4540,7 +4919,7 @@
 4. DADO token vencido CUANDO consulta ENTONCES responde 401 y vuelve a /login</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>1. Permite entrar a / sin token
 2. Guarda la contrasena en localStorage
@@ -4550,22 +4929,22 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>RF-30</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero recuperar mi clave desde /recuperar y /restablecer para volver a entrar sin ayuda del administrador.</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>1. Solicitar con correo existente devuelve 200 y crea token 32 hex
 2. Restablecer con token valido devuelve 200 y login con nueva da 200
@@ -4574,7 +4953,7 @@
 5. Correo inexistente devuelve 200 sin crear enlace</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>1. Revela si el correo existe
 2. Permite reusar el enlace mas de una vez
@@ -4584,22 +4963,22 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>RF-31</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver el dashboard con KPIs y filtros combinables para entender el gasto sin recargar la pagina.</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>1. KPIs total dinero/total/promedio se recalculan al cambiar filtro
 2. Filtros depto/modalidad/fechas son combinables y persisten
@@ -4608,7 +4987,7 @@
 5. Tab recorre select-&gt;boton-&gt;tabla-&gt;mapa sin raton</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>1. Early return if(cargando) desmonta el mapa y pierde zoom
 2. Filtros se pierden al navegar entre vistas
@@ -4618,22 +4997,22 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>RF-32</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero una tabla rapida con boton CSV para revisar miles de contratos sin que se congele y descargar lo filtrado.</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>1. Scroll mantiene 60FPS con max 50 nodos en DOM
 2. Paginacion 20/page con next/previous/count
@@ -4641,7 +5020,7 @@
 4. Filtro vacio exporta solo cabecera sin error</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>1. Renderiza todas las filas al DOM y se congela
 2. Exporta datos globales ignorando el filtro
@@ -4651,22 +5030,22 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>RF-33</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero un mapa clicable y un buscador tipo Google para filtrar por territorio o texto sin perder mis filtros.</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>1. Mapa pinta escala continua y tooltip con monto+%
 2. Clic en territorio refiltra KPIs sin borrar otros filtros
@@ -4675,7 +5054,7 @@
 5. Busqueda sin coincidencias devuelve vacio sin error</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>1. Mapa beige vacio sin colores
 2. Clic recarga la pagina o borra filtros
@@ -4685,22 +5064,22 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>RF-34</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero ver alertas y lista de entidades con umbrales editables para ajustar la deteccion sin reiniciar.</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>1. Umbrales listan valores actuales y validan rango 400 si invalido
 2. Cambio de umbral recalcula sin reinicio
@@ -4709,7 +5088,7 @@
 5. Entidad sin contratos devuelve 0 sin error</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>1. Umbral fijo no configurable
 2. Cambio exige reinicio manual
@@ -4719,22 +5098,22 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>RF-35</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Como usuario, quiero una red entidad-&gt;contratista navegable con teclado para detectar concentracion visualmente.</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>1. Grafo permite zoom/drag y destaca NIT sobre umbral
 2. Arista grosor por monto y color por modalidad
@@ -4743,12 +5122,233 @@
 5. Build minificado OK</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>1. Grafo estatico sin zoom ni drag
 2. Todas las aristas igual grosor y color
 3. Sin foco visible al navegar con teclado
 4. Solo funciona en un navegador</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>RF-36</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero crear un Radar con departamento objetivo, palabras clave y rango de cuantia para guardar mi preferencia de busqueda y recibir oportunidades automaticas.</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>1. DADO usuario autenticado, CUANDO POST /api/radares/ con {departamento_objetivo:"Boyaca", palabras_clave:"pavimento", rango_min:10000000, rango_max:50000000}, ENTONCES responde 201 con id y datos
+2. DADO palabras_clave vacias, CUANDO crea, ENTONCES responde 400
+3. DADO rango_min &gt; rango_max, ENTONCES 400
+4. DADO sin token, ENTONCES 401</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>1. Crea Radar sin usuario asociado
+2. Permite palabras_clave vacias
+3. Acepta rango_min &gt; rango_max
+4. Permite crear sin autenticacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>RF-37</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero listar mis Radares para ver y gestionar mis preferencias guardadas.</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>1. DADO usuario con 2 radares, CUANDO GET /api/radares/, ENTONCES devuelve 2 solo suyos
+2. DADO usuario sin radares, ENTONCES lista vacia count 0
+3. DADO sin token, ENTONCES 401</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>1. Devuelve radares de otros usuarios
+2. Lista vacia da error
+3. Permite listar sin auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>RF-38</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero actualizar o eliminar un Radar para ajustar mis intereses sin crear uno nuevo.</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>1. DADO usuario dueño, CUANDO PUT /api/radares/{id}/ con nuevos datos, ENTONCES 200 y actualiza
+2. DADO usuario no dueño, CUANDO PUT otro radar, ENTONCES 404
+3. DADO DELETE dueño, ENTONCES 204 y no aparece en listado</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>1. Permite editar radar ajeno
+2. DELETE no verifica pertenencia
+3. Actualiza con datos invalidos sin validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>RF-39</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero consultar mi bandeja privada de Oportunidades (mis matches) para ver contratos que coinciden con mis Radares sin buscar manualmente.</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>1. DADO Radar Boyaca+pavimento y ETL inserta contrato Boyaca pavimento 20M, CUANDO GET /api/mis-oportunidades/, ENTONCES aparece 1 con estado Nueva y contrato embebido
+2. DADO sin matches, ENTONCES lista vacia
+3. DADO sin token, ENTONCES 401
+4. Paginada con page_size 20 y count</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>1. Muestra oportunidades de otros usuarios
+2. No embebe datos de contrato
+3. Permite ver sin login
+4. No pagina</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>RF-40</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero marcar una Oportunidad como Guardada o Postulada para organizar mi flujo de trabajo.</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>1. DADO oportunidad Nueva, CUANDO PATCH {estado:"Guardada"}, ENTONCES 200 y estado cambia
+2. DADO estado invalido "X", ENTONCES 400
+3. DADO oportunidad ajena, ENTONCES 404</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>1. Permite cambiar a estado invalido
+2. Permite cambiar oportunidad ajena
+3. No valida pertenencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>RF-41</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Como contratista, quiero recibir un email cuando se cree una nueva Oportunidad que coincide con mi Radar para no revisar la bandeja a diario.</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>1. DADO se crea Oportunidad Nueva, CUANDO termina matchmaking, ENTONCES se ejecuta send_mail a usuario.email con asunto y link
+2. DADO EMAIL_BACKEND console en dev, ENTONCES imprime en consola sin error
+3. DADO fallo email, ENTONCES ETL no aborta y Oportunidad queda creada</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>1. No envia email tras crear Oportunidad
+2. Aborta ETL si email falla
+3. Envia email a usuario equivocado</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>RF-42</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Como usuario, quiero poder filtrar y crear Radares usando cualquiera de las 85 columnas del dataset (filtros elegibles) para precisar mi busqueda mas alla de depto y palabras clave.</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>1. DADO Radar con filtro {modalidad:"Licitacion publica", ciudad:"Tunja"}, CUANDO crea, ENTONCES 201 y matchmaking usa esos campos
+2. DADO campo inexistente "foo", ENTONCES 400
+3. DADO filtro por 85 cols completo, CUANDO ETL hace match, ENTONCES filtra por todos los campos elegidos con Q objects</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>1. Solo permite filtrar por depto y palabras_clave
+2. Acepta campo inexistente
+3. Ignora filtros elegibles en matchmaking</t>
         </is>
       </c>
     </row>

</xml_diff>